<commit_message>
2006 and umbral de pobreza
</commit_message>
<xml_diff>
--- a/data_externa.xlsx
+++ b/data_externa.xlsx
@@ -94,7 +94,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="79">
   <si>
     <t xml:space="preserve">Año</t>
   </si>
@@ -318,13 +318,19 @@
     <t xml:space="preserve">         --</t>
   </si>
   <si>
+    <t xml:space="preserve">Nacional IPC</t>
+  </si>
+  <si>
     <t xml:space="preserve">Encuesta condiciones de vida</t>
   </si>
   <si>
-    <t xml:space="preserve">deflactor</t>
+    <t xml:space="preserve">deflactor precios 2014</t>
   </si>
   <si>
-    <t xml:space="preserve">umbral mensual</t>
+    <t xml:space="preserve">umbral mensual precios 2014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La quinta y última ronda de la encuesta de condiciones de vida fue en 2006, de ahí en adelante justamos con la metodología del banco central</t>
   </si>
 </sst>
 </file>
@@ -497,7 +503,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -574,6 +580,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -613,6 +623,48 @@
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>1217160</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>160560</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>398160</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>32760</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="Image 1" descr=""/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7701120" y="160560"/>
+          <a:ext cx="6990120" cy="4253760"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9685,6 +9737,9 @@
       <c r="O70" s="2" t="n">
         <v>170</v>
       </c>
+      <c r="Q70" s="1" t="n">
+        <v>78.5580026568857</v>
+      </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="2" t="n">
@@ -9729,6 +9784,9 @@
       <c r="O71" s="2" t="n">
         <v>170</v>
       </c>
+      <c r="Q71" s="1" t="n">
+        <v>79.3333255724429</v>
+      </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="2" t="n">
@@ -9773,6 +9831,9 @@
       <c r="O72" s="2" t="n">
         <v>170</v>
       </c>
+      <c r="Q72" s="1" t="n">
+        <v>79.3793106370988</v>
+      </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="2" t="n">
@@ -9817,6 +9878,9 @@
       <c r="O73" s="2" t="n">
         <v>170</v>
       </c>
+      <c r="Q73" s="1" t="n">
+        <v>79.9018320639328</v>
+      </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="2" t="n">
@@ -9861,6 +9925,9 @@
       <c r="O74" s="2" t="n">
         <v>200</v>
       </c>
+      <c r="Q74" s="1" t="n">
+        <v>76.7001060910241</v>
+      </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="2" t="n">
@@ -9905,6 +9972,9 @@
       <c r="O75" s="2" t="n">
         <v>200</v>
       </c>
+      <c r="Q75" s="1" t="n">
+        <v>76.5910905819068</v>
+      </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="2" t="n">
@@ -9949,6 +10019,9 @@
       <c r="O76" s="2" t="n">
         <v>200</v>
       </c>
+      <c r="Q76" s="1" t="n">
+        <v>78.72971177482</v>
+      </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="2" t="n">
@@ -9993,6 +10066,9 @@
       <c r="O77" s="2" t="n">
         <v>200</v>
       </c>
+      <c r="Q77" s="1" t="n">
+        <v>80.4008617184761</v>
+      </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2" t="n">
@@ -10037,6 +10113,9 @@
       <c r="O78" s="2" t="n">
         <v>218</v>
       </c>
+      <c r="Q78" s="1" t="n">
+        <v>77.6887164229579</v>
+      </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="2" t="n">
@@ -10081,6 +10160,9 @@
       <c r="O79" s="2" t="n">
         <v>218</v>
       </c>
+      <c r="Q79" s="1" t="n">
+        <v>78.3304498781043</v>
+      </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="2" t="n">
@@ -10125,6 +10207,9 @@
       <c r="O80" s="2" t="n">
         <v>218</v>
       </c>
+      <c r="Q80" s="1" t="n">
+        <v>80.2472054940993</v>
+      </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="2" t="n">
@@ -10169,6 +10254,9 @@
       <c r="O81" s="2" t="n">
         <v>218</v>
       </c>
+      <c r="Q81" s="1" t="n">
+        <v>80.0487440617832</v>
+      </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="2" t="n">
@@ -10213,6 +10301,9 @@
       <c r="O82" s="2" t="n">
         <v>240</v>
       </c>
+      <c r="Q82" s="1" t="n">
+        <v>77.6249730304874</v>
+      </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="2" t="n">
@@ -10257,6 +10348,9 @@
       <c r="O83" s="2" t="n">
         <v>240</v>
       </c>
+      <c r="Q83" s="1" t="n">
+        <v>78.922062578991</v>
+      </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="2" t="n">
@@ -10301,6 +10395,9 @@
       <c r="O84" s="2" t="n">
         <v>240</v>
       </c>
+      <c r="Q84" s="1" t="n">
+        <v>80.012357407004</v>
+      </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="2" t="n">
@@ -10345,6 +10442,9 @@
       <c r="O85" s="2" t="n">
         <v>240</v>
       </c>
+      <c r="Q85" s="1" t="n">
+        <v>80.1736550181988</v>
+      </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="2" t="n">
@@ -10389,6 +10489,9 @@
       <c r="O86" s="2" t="n">
         <v>264</v>
       </c>
+      <c r="Q86" s="1" t="n">
+        <v>77.6342008561023</v>
+      </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="2" t="n">
@@ -10433,6 +10536,9 @@
       <c r="O87" s="2" t="n">
         <v>264</v>
       </c>
+      <c r="Q87" s="1" t="n">
+        <v>78.3539215544479</v>
+      </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="2" t="n">
@@ -10477,6 +10583,9 @@
       <c r="O88" s="2" t="n">
         <v>264</v>
       </c>
+      <c r="Q88" s="1" t="n">
+        <v>79.4314883699501</v>
+      </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="2" t="n">
@@ -10521,6 +10630,9 @@
       <c r="O89" s="2" t="n">
         <v>264</v>
       </c>
+      <c r="Q89" s="1" t="n">
+        <v>79.7263913317997</v>
+      </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="2" t="n">
@@ -10565,6 +10677,9 @@
       <c r="O90" s="2" t="n">
         <v>292</v>
       </c>
+      <c r="Q90" s="1" t="n">
+        <v>77.5114313879994</v>
+      </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="2" t="n">
@@ -10609,6 +10724,9 @@
       <c r="O91" s="2" t="n">
         <v>292</v>
       </c>
+      <c r="Q91" s="1" t="n">
+        <v>78.7685738034556</v>
+      </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="2" t="n">
@@ -10653,6 +10771,9 @@
       <c r="O92" s="2" t="n">
         <v>292</v>
       </c>
+      <c r="Q92" s="1" t="n">
+        <v>79.4518657001009</v>
+      </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="2" t="n">
@@ -10697,6 +10818,9 @@
       <c r="O93" s="2" t="n">
         <v>292</v>
       </c>
+      <c r="Q93" s="1" t="n">
+        <v>80.059374266261</v>
+      </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="2" t="n">
@@ -10741,6 +10865,9 @@
       <c r="O94" s="2" t="n">
         <v>318</v>
       </c>
+      <c r="Q94" s="1" t="n">
+        <v>78.3337756056933</v>
+      </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="2" t="n">
@@ -10785,6 +10912,9 @@
       <c r="O95" s="2" t="n">
         <v>318</v>
       </c>
+      <c r="Q95" s="1" t="n">
+        <v>79.2445523354866</v>
+      </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="2" t="n">
@@ -10829,6 +10959,9 @@
       <c r="O96" s="2" t="n">
         <v>318</v>
       </c>
+      <c r="Q96" s="1" t="n">
+        <v>80.0594550800498</v>
+      </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="2" t="n">
@@ -10873,6 +11006,9 @@
       <c r="O97" s="2" t="n">
         <v>318</v>
       </c>
+      <c r="Q97" s="1" t="n">
+        <v>79.8852423179184</v>
+      </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="2" t="n">
@@ -10917,6 +11053,9 @@
       <c r="O98" s="2" t="n">
         <v>340</v>
       </c>
+      <c r="Q98" s="1" t="n">
+        <v>77.8671390833756</v>
+      </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="2" t="n">
@@ -10961,6 +11100,9 @@
       <c r="O99" s="2" t="n">
         <v>340</v>
       </c>
+      <c r="Q99" s="1" t="n">
+        <v>78.8786271773628</v>
+      </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="2" t="n">
@@ -11005,6 +11147,9 @@
       <c r="O100" s="2" t="n">
         <v>340</v>
       </c>
+      <c r="Q100" s="1" t="n">
+        <v>79.5128685797242</v>
+      </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="2" t="n">
@@ -11049,6 +11194,9 @@
       <c r="O101" s="2" t="n">
         <v>340</v>
       </c>
+      <c r="Q101" s="1" t="n">
+        <v>80.1530209722584</v>
+      </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="2" t="n">
@@ -11096,6 +11244,9 @@
       <c r="O102" s="2" t="n">
         <v>354</v>
       </c>
+      <c r="Q102" s="1" t="n">
+        <v>77.8823883305729</v>
+      </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="2" t="n">
@@ -11143,6 +11294,9 @@
       <c r="O103" s="2" t="n">
         <v>354</v>
       </c>
+      <c r="Q103" s="1" t="n">
+        <v>78.2776170788467</v>
+      </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="2" t="n">
@@ -11190,6 +11344,9 @@
       <c r="O104" s="2" t="n">
         <v>354</v>
       </c>
+      <c r="Q104" s="1" t="n">
+        <v>79.8829584681759</v>
+      </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="2" t="n">
@@ -11237,6 +11394,9 @@
       <c r="O105" s="2" t="n">
         <v>354</v>
       </c>
+      <c r="Q105" s="1" t="n">
+        <v>80.6756338864045</v>
+      </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="2" t="n">
@@ -11284,6 +11444,9 @@
       <c r="O106" s="2" t="n">
         <v>366</v>
       </c>
+      <c r="Q106" s="1" t="n">
+        <v>78.4506852705083</v>
+      </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="2" t="n">
@@ -11331,6 +11494,9 @@
       <c r="O107" s="2" t="n">
         <v>366</v>
       </c>
+      <c r="Q107" s="1" t="n">
+        <v>79.0498146823104</v>
+      </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="2" t="n">
@@ -11378,6 +11544,9 @@
       <c r="O108" s="2" t="n">
         <v>366</v>
       </c>
+      <c r="Q108" s="1" t="n">
+        <v>80.068083809346</v>
+      </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="2" t="n">
@@ -11425,6 +11594,9 @@
       <c r="O109" s="2" t="n">
         <v>366</v>
       </c>
+      <c r="Q109" s="1" t="n">
+        <v>80.8915252847684</v>
+      </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="2" t="n">
@@ -11472,6 +11644,9 @@
       <c r="O110" s="2" t="n">
         <v>375</v>
       </c>
+      <c r="Q110" s="1" t="n">
+        <v>78.6242170176104</v>
+      </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="2" t="n">
@@ -11519,6 +11694,9 @@
       <c r="O111" s="2" t="n">
         <v>375</v>
       </c>
+      <c r="Q111" s="1" t="n">
+        <v>79.1721233555107</v>
+      </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="2" t="n">
@@ -11566,6 +11744,9 @@
       <c r="O112" s="2" t="n">
         <v>375</v>
       </c>
+      <c r="Q112" s="1" t="n">
+        <v>80.5987947312549</v>
+      </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="2" t="n">
@@ -11613,6 +11794,9 @@
       <c r="O113" s="2" t="n">
         <v>375</v>
       </c>
+      <c r="Q113" s="1" t="n">
+        <v>81.123565904233</v>
+      </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="2" t="n">
@@ -11660,6 +11844,9 @@
       <c r="O114" s="2" t="n">
         <v>386</v>
       </c>
+      <c r="Q114" s="1" t="n">
+        <v>78.6094904566452</v>
+      </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="2" t="n">
@@ -11707,6 +11894,9 @@
       <c r="O115" s="2" t="n">
         <v>386</v>
       </c>
+      <c r="Q115" s="1" t="n">
+        <v>79.7188863545955</v>
+      </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="2" t="n">
@@ -11754,6 +11944,9 @@
       <c r="O116" s="2" t="n">
         <v>386</v>
       </c>
+      <c r="Q116" s="1" t="n">
+        <v>80.1034446265281</v>
+      </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="2" t="n">
@@ -11801,6 +11994,9 @@
       <c r="O117" s="2" t="n">
         <v>386</v>
       </c>
+      <c r="Q117" s="1" t="n">
+        <v>80.6923164137043</v>
+      </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="2" t="n">
@@ -11848,6 +12044,9 @@
       <c r="O118" s="2" t="n">
         <v>394</v>
       </c>
+      <c r="Q118" s="1" t="n">
+        <v>78.7032739397182</v>
+      </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="2" t="n">
@@ -11895,6 +12094,9 @@
       <c r="O119" s="2" t="n">
         <v>394</v>
       </c>
+      <c r="Q119" s="1" t="n">
+        <v>79.5614926013539</v>
+      </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="2" t="n">
@@ -11942,6 +12144,9 @@
       <c r="O120" s="2" t="n">
         <v>394</v>
       </c>
+      <c r="Q120" s="1" t="n">
+        <v>80.1589598599</v>
+      </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="2" t="n">
@@ -11989,6 +12194,9 @@
       <c r="O121" s="2" t="n">
         <v>394</v>
       </c>
+      <c r="Q121" s="1" t="n">
+        <v>80.8245161035507</v>
+      </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="2" t="n">
@@ -12036,6 +12244,9 @@
       <c r="O122" s="2" t="n">
         <v>400</v>
       </c>
+      <c r="Q122" s="1" t="n">
+        <v>78.919576103865</v>
+      </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="2" t="n">
@@ -12083,6 +12294,9 @@
       <c r="O123" s="2" t="n">
         <v>400</v>
       </c>
+      <c r="Q123" s="1" t="n">
+        <v>78.9602207181246</v>
+      </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="2" t="n">
@@ -12130,6 +12344,9 @@
       <c r="O124" s="2" t="n">
         <v>400</v>
       </c>
+      <c r="Q124" s="1" t="n">
+        <v>81.2706714423633</v>
+      </c>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="2" t="n">
@@ -12177,6 +12394,9 @@
       <c r="O125" s="2" t="n">
         <v>400</v>
       </c>
+      <c r="Q125" s="1" t="n">
+        <v>81.1657430331955</v>
+      </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="2" t="n">
@@ -12224,6 +12444,9 @@
       <c r="O126" s="2" t="n">
         <v>400</v>
       </c>
+      <c r="Q126" s="1" t="n">
+        <v>78.7141199098841</v>
+      </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="2" t="n">
@@ -12271,6 +12494,9 @@
       <c r="O127" s="2" t="n">
         <v>400</v>
       </c>
+      <c r="Q127" s="1" t="n">
+        <v>79.1238681762521</v>
+      </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="2" t="n">
@@ -12318,6 +12544,9 @@
       <c r="O128" s="2" t="n">
         <v>400</v>
       </c>
+      <c r="Q128" s="1" t="n">
+        <v>79.7392310959229</v>
+      </c>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="2" t="n">
@@ -12365,6 +12594,9 @@
       <c r="O129" s="2" t="n">
         <v>400</v>
       </c>
+      <c r="Q129" s="1" t="n">
+        <v>80.4092251038578</v>
+      </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="2" t="n">
@@ -12412,6 +12644,9 @@
       <c r="O130" s="2" t="n">
         <v>425</v>
       </c>
+      <c r="Q130" s="1" t="n">
+        <v>78.0347697832917</v>
+      </c>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="2" t="n">
@@ -12459,6 +12694,9 @@
       <c r="O131" s="2" t="n">
         <v>425</v>
       </c>
+      <c r="Q131" s="1" t="n">
+        <v>78.4613499982757</v>
+      </c>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="2" t="n">
@@ -12506,6 +12744,9 @@
       <c r="O132" s="2" t="n">
         <v>425</v>
       </c>
+      <c r="Q132" s="1" t="n">
+        <v>79.4246182804694</v>
+      </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="2" t="n">
@@ -12553,6 +12794,9 @@
       <c r="O133" s="2" t="n">
         <v>425</v>
       </c>
+      <c r="Q133" s="1" t="n">
+        <v>80.4956142277642</v>
+      </c>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="2" t="n">
@@ -12600,6 +12844,9 @@
       <c r="O134" s="2" t="n">
         <v>450</v>
       </c>
+      <c r="Q134" s="1" t="n">
+        <v>78.6761103637299</v>
+      </c>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="2" t="n">
@@ -12647,6 +12894,9 @@
       <c r="O135" s="2" t="n">
         <v>450</v>
       </c>
+      <c r="Q135" s="1" t="n">
+        <v>79.1721687083274</v>
+      </c>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="2" t="n">
@@ -12694,6 +12944,9 @@
       <c r="O136" s="2" t="n">
         <v>450</v>
       </c>
+      <c r="Q136" s="1" t="n">
+        <v>79.2260952598721</v>
+      </c>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="2" t="n">
@@ -12741,6 +12994,9 @@
       <c r="O137" s="2" t="n">
         <v>450</v>
       </c>
+      <c r="Q137" s="1" t="n">
+        <v>81.0356815331653</v>
+      </c>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="2" t="n">
@@ -12788,6 +13044,9 @@
       <c r="O138" s="2" t="n">
         <v>460</v>
       </c>
+      <c r="Q138" s="1" t="n">
+        <v>78.7729090748131</v>
+      </c>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="2" t="n">
@@ -12835,6 +13094,9 @@
       <c r="O139" s="2" t="n">
         <v>460</v>
       </c>
+      <c r="Q139" s="1" t="n">
+        <v>78.650586183592</v>
+      </c>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="2" t="n">
@@ -12882,6 +13144,9 @@
       <c r="O140" s="2" t="n">
         <v>460</v>
       </c>
+      <c r="Q140" s="1" t="n">
+        <v>79.792911130647</v>
+      </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="2" t="n">
@@ -12928,6 +13193,9 @@
       </c>
       <c r="O141" s="2" t="n">
         <v>460</v>
+      </c>
+      <c r="Q141" s="1" t="n">
+        <v>81.2723496253218</v>
       </c>
     </row>
   </sheetData>
@@ -30141,7 +30409,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F141"/>
+  <dimension ref="A1:G141"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="17.71"/>
@@ -30159,16 +30427,16 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>74</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30306,7 +30574,7 @@
       </c>
       <c r="F7" s="2" t="n">
         <f aca="false">E7*D7</f>
-        <v>928.537384529419</v>
+        <v>928.537384529417</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31693,6 +31961,21 @@
       <c r="C70" s="2" t="n">
         <v>71.3039474435275</v>
       </c>
+      <c r="D70" s="19" t="n">
+        <f aca="false">$D$69*(C69/AVERAGE($C$66:$C$69))</f>
+        <v>57.1097311275349</v>
+      </c>
+      <c r="E70" s="2" t="n">
+        <f aca="false">$C$98/C70</f>
+        <v>1.37556246730445</v>
+      </c>
+      <c r="F70" s="2" t="n">
+        <f aca="false">E70*D70</f>
+        <v>78.5580026568857</v>
+      </c>
+      <c r="G70" s="2" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="2" t="n">
@@ -31704,6 +31987,18 @@
       <c r="C71" s="2" t="n">
         <v>71.4653187847975</v>
       </c>
+      <c r="D71" s="19" t="n">
+        <f aca="false">$D$69*(C70/AVERAGE($C$66:$C$69))</f>
+        <v>57.3428172491019</v>
+      </c>
+      <c r="E71" s="2" t="n">
+        <f aca="false">$C$99/C71</f>
+        <v>1.38349194159423</v>
+      </c>
+      <c r="F71" s="2" t="n">
+        <f aca="false">E71*D71</f>
+        <v>79.3333255724429</v>
+      </c>
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="2" t="n">
@@ -31715,6 +32010,18 @@
       <c r="C72" s="2" t="n">
         <v>72.1618914219933</v>
       </c>
+      <c r="D72" s="19" t="n">
+        <f aca="false">$D$69*(C71/AVERAGE($C$66:$C$69))</f>
+        <v>57.4725924952623</v>
+      </c>
+      <c r="E72" s="2" t="n">
+        <f aca="false">$C$100/C72</f>
+        <v>1.38116808709547</v>
+      </c>
+      <c r="F72" s="2" t="n">
+        <f aca="false">E72*D72</f>
+        <v>79.3793106370988</v>
+      </c>
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="2" t="n">
@@ -31726,6 +32033,18 @@
       <c r="C73" s="2" t="n">
         <v>72.9978954822526</v>
       </c>
+      <c r="D73" s="19" t="n">
+        <f aca="false">$D$69*(C72/AVERAGE($C$66:$C$69))</f>
+        <v>58.0327779950494</v>
+      </c>
+      <c r="E73" s="2" t="n">
+        <f aca="false">$C$101/C73</f>
+        <v>1.37683968998949</v>
+      </c>
+      <c r="F73" s="2" t="n">
+        <f aca="false">E73*D73</f>
+        <v>79.9018320639328</v>
+      </c>
     </row>
     <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="2" t="n">
@@ -31737,6 +32056,18 @@
       <c r="C74" s="2" t="n">
         <v>75.0712622958227</v>
       </c>
+      <c r="D74" s="19" t="n">
+        <f aca="false">$D$69*(C73/AVERAGE($C$66:$C$69))</f>
+        <v>58.7050946025545</v>
+      </c>
+      <c r="E74" s="2" t="n">
+        <f aca="false">$C$98/C74</f>
+        <v>1.30653236504088</v>
+      </c>
+      <c r="F74" s="2" t="n">
+        <f aca="false">E74*D74</f>
+        <v>76.7001060910241</v>
+      </c>
     </row>
     <row r="75" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="2" t="n">
@@ -31748,6 +32079,18 @@
       <c r="C75" s="2" t="n">
         <v>77.935062259733</v>
       </c>
+      <c r="D75" s="19" t="n">
+        <f aca="false">$D$69*(C74/AVERAGE($C$66:$C$69))</f>
+        <v>60.3725015069908</v>
+      </c>
+      <c r="E75" s="2" t="n">
+        <f aca="false">$C$99/C75</f>
+        <v>1.26864199213342</v>
+      </c>
+      <c r="F75" s="2" t="n">
+        <f aca="false">E75*D75</f>
+        <v>76.5910905819068</v>
+      </c>
     </row>
     <row r="76" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="2" t="n">
@@ -31759,6 +32102,18 @@
       <c r="C76" s="2" t="n">
         <v>79.3440054454324</v>
       </c>
+      <c r="D76" s="19" t="n">
+        <f aca="false">$D$69*(C75/AVERAGE($C$66:$C$69))</f>
+        <v>62.6755767764007</v>
+      </c>
+      <c r="E76" s="2" t="n">
+        <f aca="false">$C$100/C76</f>
+        <v>1.25614658570584</v>
+      </c>
+      <c r="F76" s="2" t="n">
+        <f aca="false">E76*D76</f>
+        <v>78.72971177482</v>
+      </c>
     </row>
     <row r="77" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="2" t="n">
@@ -31770,6 +32125,18 @@
       <c r="C77" s="2" t="n">
         <v>79.7650398334914</v>
       </c>
+      <c r="D77" s="19" t="n">
+        <f aca="false">$D$69*(C76/AVERAGE($C$66:$C$69))</f>
+        <v>63.8086524967305</v>
+      </c>
+      <c r="E77" s="2" t="n">
+        <f aca="false">$C$101/C77</f>
+        <v>1.26003071013913</v>
+      </c>
+      <c r="F77" s="2" t="n">
+        <f aca="false">E77*D77</f>
+        <v>80.4008617184761</v>
+      </c>
     </row>
     <row r="78" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2" t="n">
@@ -31781,6 +32148,18 @@
       <c r="C78" s="2" t="n">
         <v>80.9867523690246</v>
       </c>
+      <c r="D78" s="19" t="n">
+        <f aca="false">$D$69*(C77/AVERAGE($C$66:$C$69))</f>
+        <v>64.1472494305002</v>
+      </c>
+      <c r="E78" s="2" t="n">
+        <f aca="false">$C$98/C78</f>
+        <v>1.21109972933647</v>
+      </c>
+      <c r="F78" s="2" t="n">
+        <f aca="false">E78*D78</f>
+        <v>77.6887164229579</v>
+      </c>
     </row>
     <row r="79" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="2" t="n">
@@ -31792,6 +32171,18 @@
       <c r="C79" s="2" t="n">
         <v>82.2092686539893</v>
       </c>
+      <c r="D79" s="19" t="n">
+        <f aca="false">$D$69*(C78/AVERAGE($C$66:$C$69))</f>
+        <v>65.1297537821913</v>
+      </c>
+      <c r="E79" s="2" t="n">
+        <f aca="false">$C$99/C79</f>
+        <v>1.20268303393345</v>
+      </c>
+      <c r="F79" s="2" t="n">
+        <f aca="false">E79*D79</f>
+        <v>78.3304498781043</v>
+      </c>
     </row>
     <row r="80" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="2" t="n">
@@ -31803,6 +32194,18 @@
       <c r="C80" s="2" t="n">
         <v>82.1127812983064</v>
       </c>
+      <c r="D80" s="19" t="n">
+        <f aca="false">$D$69*(C79/AVERAGE($C$66:$C$69))</f>
+        <v>66.1129045112347</v>
+      </c>
+      <c r="E80" s="2" t="n">
+        <f aca="false">$C$100/C80</f>
+        <v>1.21379034981685</v>
+      </c>
+      <c r="F80" s="2" t="n">
+        <f aca="false">E80*D80</f>
+        <v>80.2472054940993</v>
+      </c>
     </row>
     <row r="81" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="2" t="n">
@@ -31814,6 +32217,18 @@
       <c r="C81" s="2" t="n">
         <v>82.9116216304853</v>
       </c>
+      <c r="D81" s="19" t="n">
+        <f aca="false">$D$69*(C80/AVERAGE($C$66:$C$69))</f>
+        <v>66.0353091325475</v>
+      </c>
+      <c r="E81" s="2" t="n">
+        <f aca="false">$C$101/C81</f>
+        <v>1.21221124143006</v>
+      </c>
+      <c r="F81" s="2" t="n">
+        <f aca="false">E81*D81</f>
+        <v>80.0487440617832</v>
+      </c>
     </row>
     <row r="82" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="2" t="n">
@@ -31825,6 +32240,18 @@
       <c r="C82" s="2" t="n">
         <v>84.2506558899935</v>
       </c>
+      <c r="D82" s="19" t="n">
+        <f aca="false">$D$69*(C81/AVERAGE($C$66:$C$69))</f>
+        <v>66.677738574699</v>
+      </c>
+      <c r="E82" s="2" t="n">
+        <f aca="false">$C$98/C82</f>
+        <v>1.16418124984134</v>
+      </c>
+      <c r="F82" s="2" t="n">
+        <f aca="false">E82*D82</f>
+        <v>77.6249730304874</v>
+      </c>
     </row>
     <row r="83" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="2" t="n">
@@ -31836,6 +32263,18 @@
       <c r="C83" s="2" t="n">
         <v>84.8813514323926</v>
       </c>
+      <c r="D83" s="19" t="n">
+        <f aca="false">$D$69*(C82/AVERAGE($C$66:$C$69))</f>
+        <v>67.7545933574455</v>
+      </c>
+      <c r="E83" s="2" t="n">
+        <f aca="false">$C$99/C83</f>
+        <v>1.16482231931687</v>
+      </c>
+      <c r="F83" s="2" t="n">
+        <f aca="false">E83*D83</f>
+        <v>78.922062578991</v>
+      </c>
     </row>
     <row r="84" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="2" t="n">
@@ -31847,6 +32286,18 @@
       <c r="C84" s="2" t="n">
         <v>85.0305748011699</v>
       </c>
+      <c r="D84" s="19" t="n">
+        <f aca="false">$D$69*(C83/AVERAGE($C$66:$C$69))</f>
+        <v>68.2618003287883</v>
+      </c>
+      <c r="E84" s="2" t="n">
+        <f aca="false">$C$100/C84</f>
+        <v>1.17213957179005</v>
+      </c>
+      <c r="F84" s="2" t="n">
+        <f aca="false">E84*D84</f>
+        <v>80.012357407004</v>
+      </c>
     </row>
     <row r="85" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="2" t="n">
@@ -31858,6 +32309,18 @@
       <c r="C85" s="2" t="n">
         <v>85.7240342210823</v>
       </c>
+      <c r="D85" s="19" t="n">
+        <f aca="false">$D$69*(C84/AVERAGE($C$66:$C$69))</f>
+        <v>68.381806144341</v>
+      </c>
+      <c r="E85" s="2" t="n">
+        <f aca="false">$C$101/C85</f>
+        <v>1.17244131939083</v>
+      </c>
+      <c r="F85" s="2" t="n">
+        <f aca="false">E85*D85</f>
+        <v>80.1736550181988</v>
+      </c>
     </row>
     <row r="86" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="2" t="n">
@@ -31869,6 +32332,18 @@
       <c r="C86" s="2" t="n">
         <v>87.0981353694548</v>
       </c>
+      <c r="D86" s="19" t="n">
+        <f aca="false">$D$69*(C85/AVERAGE($C$66:$C$69))</f>
+        <v>68.9394879868112</v>
+      </c>
+      <c r="E86" s="2" t="n">
+        <f aca="false">$C$98/C86</f>
+        <v>1.12612093769763</v>
+      </c>
+      <c r="F86" s="2" t="n">
+        <f aca="false">E86*D86</f>
+        <v>77.6342008561023</v>
+      </c>
     </row>
     <row r="87" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="2" t="n">
@@ -31880,6 +32355,18 @@
       <c r="C87" s="2" t="n">
         <v>88.3864196428003</v>
       </c>
+      <c r="D87" s="19" t="n">
+        <f aca="false">$D$69*(C86/AVERAGE($C$66:$C$69))</f>
+        <v>70.0445436514406</v>
+      </c>
+      <c r="E87" s="2" t="n">
+        <f aca="false">$C$99/C87</f>
+        <v>1.11862990990928</v>
+      </c>
+      <c r="F87" s="2" t="n">
+        <f aca="false">E87*D87</f>
+        <v>78.3539215544479</v>
+      </c>
     </row>
     <row r="88" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="2" t="n">
@@ -31891,6 +32378,18 @@
       <c r="C88" s="2" t="n">
         <v>89.1892962435327</v>
       </c>
+      <c r="D88" s="19" t="n">
+        <f aca="false">$D$69*(C87/AVERAGE($C$66:$C$69))</f>
+        <v>71.0805851652691</v>
+      </c>
+      <c r="E88" s="2" t="n">
+        <f aca="false">$C$100/C88</f>
+        <v>1.11748500923655</v>
+      </c>
+      <c r="F88" s="2" t="n">
+        <f aca="false">E88*D88</f>
+        <v>79.4314883699501</v>
+      </c>
     </row>
     <row r="89" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="2" t="n">
@@ -31902,6 +32401,18 @@
       <c r="C89" s="2" t="n">
         <v>90.421102737221</v>
       </c>
+      <c r="D89" s="19" t="n">
+        <f aca="false">$D$69*(C88/AVERAGE($C$66:$C$69))</f>
+        <v>71.7262605849343</v>
+      </c>
+      <c r="E89" s="2" t="n">
+        <f aca="false">$C$101/C89</f>
+        <v>1.11153698354861</v>
+      </c>
+      <c r="F89" s="2" t="n">
+        <f aca="false">E89*D89</f>
+        <v>79.7263913317997</v>
+      </c>
     </row>
     <row r="90" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="2" t="n">
@@ -31913,6 +32424,18 @@
       <c r="C90" s="2" t="n">
         <v>92.0160074979537</v>
       </c>
+      <c r="D90" s="19" t="n">
+        <f aca="false">$D$69*(C89/AVERAGE($C$66:$C$69))</f>
+        <v>72.7168825236392</v>
+      </c>
+      <c r="E90" s="2" t="n">
+        <f aca="false">$C$98/C90</f>
+        <v>1.06593446663231</v>
+      </c>
+      <c r="F90" s="2" t="n">
+        <f aca="false">E90*D90</f>
+        <v>77.5114313879994</v>
+      </c>
     </row>
     <row r="91" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="2" t="n">
@@ -31924,6 +32447,18 @@
       <c r="C91" s="2" t="n">
         <v>92.8854790448768</v>
       </c>
+      <c r="D91" s="19" t="n">
+        <f aca="false">$D$69*(C90/AVERAGE($C$66:$C$69))</f>
+        <v>73.9995090191338</v>
+      </c>
+      <c r="E91" s="2" t="n">
+        <f aca="false">$C$99/C91</f>
+        <v>1.0644472490093</v>
+      </c>
+      <c r="F91" s="2" t="n">
+        <f aca="false">E91*D91</f>
+        <v>78.7685738034556</v>
+      </c>
     </row>
     <row r="92" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="2" t="n">
@@ -31935,6 +32470,18 @@
       <c r="C92" s="2" t="n">
         <v>93.7051846964094</v>
       </c>
+      <c r="D92" s="19" t="n">
+        <f aca="false">$D$69*(C91/AVERAGE($C$66:$C$69))</f>
+        <v>74.6987402651737</v>
+      </c>
+      <c r="E92" s="2" t="n">
+        <f aca="false">$C$100/C92</f>
+        <v>1.06363059695591</v>
+      </c>
+      <c r="F92" s="2" t="n">
+        <f aca="false">E92*D92</f>
+        <v>79.4518657001009</v>
+      </c>
     </row>
     <row r="93" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="2" t="n">
@@ -31946,6 +32493,18 @@
       <c r="C93" s="2" t="n">
         <v>94.604239466372</v>
       </c>
+      <c r="D93" s="19" t="n">
+        <f aca="false">$D$69*(C92/AVERAGE($C$66:$C$69))</f>
+        <v>75.3579496506165</v>
+      </c>
+      <c r="E93" s="2" t="n">
+        <f aca="false">$C$101/C93</f>
+        <v>1.06238790515721</v>
+      </c>
+      <c r="F93" s="2" t="n">
+        <f aca="false">E93*D93</f>
+        <v>80.059374266261</v>
+      </c>
     </row>
     <row r="94" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="2" t="n">
@@ -31957,6 +32516,18 @@
       <c r="C94" s="2" t="n">
         <v>95.2622604561851</v>
       </c>
+      <c r="D94" s="19" t="n">
+        <f aca="false">$D$69*(C93/AVERAGE($C$66:$C$69))</f>
+        <v>76.0809718004312</v>
+      </c>
+      <c r="E94" s="2" t="n">
+        <f aca="false">$C$98/C94</f>
+        <v>1.02961060764538</v>
+      </c>
+      <c r="F94" s="2" t="n">
+        <f aca="false">E94*D94</f>
+        <v>78.3337756056933</v>
+      </c>
     </row>
     <row r="95" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="2" t="n">
@@ -31968,6 +32539,18 @@
       <c r="C95" s="2" t="n">
         <v>95.5848114857496</v>
       </c>
+      <c r="D95" s="19" t="n">
+        <f aca="false">$D$69*(C94/AVERAGE($C$66:$C$69))</f>
+        <v>76.6101539666053</v>
+      </c>
+      <c r="E95" s="2" t="n">
+        <f aca="false">$C$99/C95</f>
+        <v>1.03438706532335</v>
+      </c>
+      <c r="F95" s="2" t="n">
+        <f aca="false">E95*D95</f>
+        <v>79.2445523354866</v>
+      </c>
     </row>
     <row r="96" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="2" t="n">
@@ -31979,6 +32562,18 @@
       <c r="C96" s="2" t="n">
         <v>95.696521940927</v>
       </c>
+      <c r="D96" s="19" t="n">
+        <f aca="false">$D$69*(C95/AVERAGE($C$66:$C$69))</f>
+        <v>76.869550331112</v>
+      </c>
+      <c r="E96" s="2" t="n">
+        <f aca="false">$C$100/C96</f>
+        <v>1.04149763768875</v>
+      </c>
+      <c r="F96" s="2" t="n">
+        <f aca="false">E96*D96</f>
+        <v>80.0594550800498</v>
+      </c>
     </row>
     <row r="97" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="2" t="n">
@@ -31990,6 +32585,18 @@
       <c r="C97" s="2" t="n">
         <v>96.8252809878436</v>
       </c>
+      <c r="D97" s="19" t="n">
+        <f aca="false">$D$69*(C96/AVERAGE($C$66:$C$69))</f>
+        <v>76.9593881654216</v>
+      </c>
+      <c r="E97" s="2" t="n">
+        <f aca="false">$C$101/C97</f>
+        <v>1.03801815765749</v>
+      </c>
+      <c r="F97" s="2" t="n">
+        <f aca="false">E97*D97</f>
+        <v>79.8852423179184</v>
+      </c>
     </row>
     <row r="98" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="2" t="n">
@@ -32001,6 +32608,18 @@
       <c r="C98" s="2" t="n">
         <v>98.0830338739655</v>
       </c>
+      <c r="D98" s="19" t="n">
+        <f aca="false">$D$69*(C97/AVERAGE($C$66:$C$69))</f>
+        <v>77.8671390833756</v>
+      </c>
+      <c r="E98" s="2" t="n">
+        <f aca="false">$C$98/C98</f>
+        <v>1</v>
+      </c>
+      <c r="F98" s="2" t="n">
+        <f aca="false">E98*D98</f>
+        <v>77.8671390833756</v>
+      </c>
     </row>
     <row r="99" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="2" t="n">
@@ -32012,6 +32631,18 @@
       <c r="C99" s="2" t="n">
         <v>98.8716926422298</v>
       </c>
+      <c r="D99" s="19" t="n">
+        <f aca="false">$D$69*(C98/AVERAGE($C$66:$C$69))</f>
+        <v>78.8786271773628</v>
+      </c>
+      <c r="E99" s="2" t="n">
+        <f aca="false">$C$99/C99</f>
+        <v>1</v>
+      </c>
+      <c r="F99" s="2" t="n">
+        <f aca="false">E99*D99</f>
+        <v>78.8786271773628</v>
+      </c>
     </row>
     <row r="100" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="2" t="n">
@@ -32023,6 +32654,18 @@
       <c r="C100" s="2" t="n">
         <v>99.6677015365054</v>
       </c>
+      <c r="D100" s="19" t="n">
+        <f aca="false">$D$69*(C99/AVERAGE($C$66:$C$69))</f>
+        <v>79.5128685797242</v>
+      </c>
+      <c r="E100" s="2" t="n">
+        <f aca="false">$C$100/C100</f>
+        <v>1</v>
+      </c>
+      <c r="F100" s="2" t="n">
+        <f aca="false">E100*D100</f>
+        <v>79.5128685797242</v>
+      </c>
     </row>
     <row r="101" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="2" t="n">
@@ -32034,6 +32677,18 @@
       <c r="C101" s="2" t="n">
         <v>100.50639978567</v>
       </c>
+      <c r="D101" s="19" t="n">
+        <f aca="false">$D$69*(C100/AVERAGE($C$66:$C$69))</f>
+        <v>80.1530209722584</v>
+      </c>
+      <c r="E101" s="2" t="n">
+        <f aca="false">$C$101/C101</f>
+        <v>1</v>
+      </c>
+      <c r="F101" s="2" t="n">
+        <f aca="false">E101*D101</f>
+        <v>80.1530209722584</v>
+      </c>
     </row>
     <row r="102" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="2" t="n">
@@ -32045,6 +32700,18 @@
       <c r="C102" s="2" t="n">
         <v>101.792035498233</v>
       </c>
+      <c r="D102" s="19" t="n">
+        <f aca="false">$D$69*(C101/AVERAGE($C$66:$C$69))</f>
+        <v>80.8275042533849</v>
+      </c>
+      <c r="E102" s="2" t="n">
+        <f aca="false">$C$98/C102</f>
+        <v>0.963562948651991</v>
+      </c>
+      <c r="F102" s="2" t="n">
+        <f aca="false">E102*D102</f>
+        <v>77.8823883305729</v>
+      </c>
     </row>
     <row r="103" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="2" t="n">
@@ -32056,6 +32723,18 @@
       <c r="C103" s="2" t="n">
         <v>103.398353744992</v>
       </c>
+      <c r="D103" s="19" t="n">
+        <f aca="false">$D$69*(C102/AVERAGE($C$66:$C$69))</f>
+        <v>81.8614157878453</v>
+      </c>
+      <c r="E103" s="2" t="n">
+        <f aca="false">$C$99/C103</f>
+        <v>0.956221149188447</v>
+      </c>
+      <c r="F103" s="2" t="n">
+        <f aca="false">E103*D103</f>
+        <v>78.2776170788467</v>
+      </c>
     </row>
     <row r="104" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="2" t="n">
@@ -32067,6 +32746,18 @@
       <c r="C104" s="2" t="n">
         <v>103.747915389501</v>
       </c>
+      <c r="D104" s="19" t="n">
+        <f aca="false">$D$69*(C103/AVERAGE($C$66:$C$69))</f>
+        <v>83.153221038049</v>
+      </c>
+      <c r="E104" s="2" t="n">
+        <f aca="false">$C$100/C104</f>
+        <v>0.960671847355417</v>
+      </c>
+      <c r="F104" s="2" t="n">
+        <f aca="false">E104*D104</f>
+        <v>79.8829584681759</v>
+      </c>
     </row>
     <row r="105" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="2" t="n">
@@ -32078,6 +32769,18 @@
       <c r="C105" s="2" t="n">
         <v>103.943218893479</v>
       </c>
+      <c r="D105" s="19" t="n">
+        <f aca="false">$D$69*(C104/AVERAGE($C$66:$C$69))</f>
+        <v>83.4343394083083</v>
+      </c>
+      <c r="E105" s="2" t="n">
+        <f aca="false">$C$101/C105</f>
+        <v>0.966935610187991</v>
+      </c>
+      <c r="F105" s="2" t="n">
+        <f aca="false">E105*D105</f>
+        <v>80.6756338864045</v>
+      </c>
     </row>
     <row r="106" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="2" t="n">
@@ -32089,6 +32792,18 @@
       <c r="C106" s="2" t="n">
         <v>104.510220432656</v>
       </c>
+      <c r="D106" s="19" t="n">
+        <f aca="false">$D$69*(C105/AVERAGE($C$66:$C$69))</f>
+        <v>83.5914029866689</v>
+      </c>
+      <c r="E106" s="2" t="n">
+        <f aca="false">$C$98/C106</f>
+        <v>0.938501837120973</v>
+      </c>
+      <c r="F106" s="2" t="n">
+        <f aca="false">E106*D106</f>
+        <v>78.4506852705083</v>
+      </c>
     </row>
     <row r="107" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="2" t="n">
@@ -32100,6 +32815,18 @@
       <c r="C107" s="2" t="n">
         <v>105.122414972079</v>
       </c>
+      <c r="D107" s="19" t="n">
+        <f aca="false">$D$69*(C106/AVERAGE($C$66:$C$69))</f>
+        <v>84.0473870774058</v>
+      </c>
+      <c r="E107" s="2" t="n">
+        <f aca="false">$C$99/C107</f>
+        <v>0.940538634586074</v>
+      </c>
+      <c r="F107" s="2" t="n">
+        <f aca="false">E107*D107</f>
+        <v>79.0498146823104</v>
+      </c>
     </row>
     <row r="108" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="2" t="n">
@@ -32111,6 +32838,18 @@
       <c r="C108" s="2" t="n">
         <v>105.233930063504</v>
       </c>
+      <c r="D108" s="19" t="n">
+        <f aca="false">$D$69*(C107/AVERAGE($C$66:$C$69))</f>
+        <v>84.5397154947467</v>
+      </c>
+      <c r="E108" s="2" t="n">
+        <f aca="false">$C$100/C108</f>
+        <v>0.947106142252412</v>
+      </c>
+      <c r="F108" s="2" t="n">
+        <f aca="false">E108*D108</f>
+        <v>80.068083809346</v>
+      </c>
     </row>
     <row r="109" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="2" t="n">
@@ -32122,6 +32861,18 @@
       <c r="C109" s="2" t="n">
         <v>105.150643406274</v>
       </c>
+      <c r="D109" s="19" t="n">
+        <f aca="false">$D$69*(C108/AVERAGE($C$66:$C$69))</f>
+        <v>84.629396217026</v>
+      </c>
+      <c r="E109" s="2" t="n">
+        <f aca="false">$C$101/C109</f>
+        <v>0.955832475483199</v>
+      </c>
+      <c r="F109" s="2" t="n">
+        <f aca="false">E109*D109</f>
+        <v>80.8915252847684</v>
+      </c>
     </row>
     <row r="110" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="2" t="n">
@@ -32133,6 +32884,18 @@
       <c r="C110" s="2" t="n">
         <v>105.490887074215</v>
       </c>
+      <c r="D110" s="19" t="n">
+        <f aca="false">$D$69*(C109/AVERAGE($C$66:$C$69))</f>
+        <v>84.5624168738611</v>
+      </c>
+      <c r="E110" s="2" t="n">
+        <f aca="false">$C$98/C110</f>
+        <v>0.92977731626204</v>
+      </c>
+      <c r="F110" s="2" t="n">
+        <f aca="false">E110*D110</f>
+        <v>78.6242170176104</v>
+      </c>
     </row>
     <row r="111" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="2" t="n">
@@ -32144,6 +32907,18 @@
       <c r="C111" s="2" t="n">
         <v>105.944904403107</v>
       </c>
+      <c r="D111" s="19" t="n">
+        <f aca="false">$D$69*(C110/AVERAGE($C$66:$C$69))</f>
+        <v>84.8360417034872</v>
+      </c>
+      <c r="E111" s="2" t="n">
+        <f aca="false">$C$99/C111</f>
+        <v>0.933236885712176</v>
+      </c>
+      <c r="F111" s="2" t="n">
+        <f aca="false">E111*D111</f>
+        <v>79.1721233555107</v>
+      </c>
     </row>
     <row r="112" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="2" t="n">
@@ -32155,6 +32930,18 @@
       <c r="C112" s="2" t="n">
         <v>105.358947026948</v>
       </c>
+      <c r="D112" s="19" t="n">
+        <f aca="false">$D$69*(C111/AVERAGE($C$66:$C$69))</f>
+        <v>85.201163602793</v>
+      </c>
+      <c r="E112" s="2" t="n">
+        <f aca="false">$C$100/C112</f>
+        <v>0.945982323750949</v>
+      </c>
+      <c r="F112" s="2" t="n">
+        <f aca="false">E112*D112</f>
+        <v>80.5987947312549</v>
+      </c>
     </row>
     <row r="113" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="2" t="n">
@@ -32166,6 +32953,18 @@
       <c r="C113" s="2" t="n">
         <v>104.974437995069</v>
       </c>
+      <c r="D113" s="19" t="n">
+        <f aca="false">$D$69*(C112/AVERAGE($C$66:$C$69))</f>
+        <v>84.7299351793812</v>
+      </c>
+      <c r="E113" s="2" t="n">
+        <f aca="false">$C$101/C113</f>
+        <v>0.957436893259587</v>
+      </c>
+      <c r="F113" s="2" t="n">
+        <f aca="false">E113*D113</f>
+        <v>81.123565904233</v>
+      </c>
     </row>
     <row r="114" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="2" t="n">
@@ -32177,6 +32976,18 @@
       <c r="C114" s="2" t="n">
         <v>105.333840858986</v>
       </c>
+      <c r="D114" s="19" t="n">
+        <f aca="false">$D$69*(C113/AVERAGE($C$66:$C$69))</f>
+        <v>84.420712030647</v>
+      </c>
+      <c r="E114" s="2" t="n">
+        <f aca="false">$C$98/C114</f>
+        <v>0.931163556499118</v>
+      </c>
+      <c r="F114" s="2" t="n">
+        <f aca="false">E114*D114</f>
+        <v>78.6094904566452</v>
+      </c>
     </row>
     <row r="115" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="2" t="n">
@@ -32188,6 +32999,18 @@
       <c r="C115" s="2" t="n">
         <v>105.061626274654</v>
       </c>
+      <c r="D115" s="19" t="n">
+        <f aca="false">$D$69*(C114/AVERAGE($C$66:$C$69))</f>
+        <v>84.7097447347721</v>
+      </c>
+      <c r="E115" s="2" t="n">
+        <f aca="false">$C$99/C115</f>
+        <v>0.941082830602276</v>
+      </c>
+      <c r="F115" s="2" t="n">
+        <f aca="false">E115*D115</f>
+        <v>79.7188863545955</v>
+      </c>
     </row>
     <row r="116" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="2" t="n">
@@ -32199,6 +33022,18 @@
       <c r="C116" s="2" t="n">
         <v>105.12664933991</v>
       </c>
+      <c r="D116" s="19" t="n">
+        <f aca="false">$D$69*(C115/AVERAGE($C$66:$C$69))</f>
+        <v>84.4908290685076</v>
+      </c>
+      <c r="E116" s="2" t="n">
+        <f aca="false">$C$100/C116</f>
+        <v>0.94807265486267</v>
+      </c>
+      <c r="F116" s="2" t="n">
+        <f aca="false">E116*D116</f>
+        <v>80.1034446265281</v>
+      </c>
     </row>
     <row r="117" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="2" t="n">
@@ -32210,6 +33045,18 @@
       <c r="C117" s="2" t="n">
         <v>105.30277322938</v>
       </c>
+      <c r="D117" s="19" t="n">
+        <f aca="false">$D$69*(C116/AVERAGE($C$66:$C$69))</f>
+        <v>84.5431207842069</v>
+      </c>
+      <c r="E117" s="2" t="n">
+        <f aca="false">$C$101/C117</f>
+        <v>0.954451594230457</v>
+      </c>
+      <c r="F117" s="2" t="n">
+        <f aca="false">E117*D117</f>
+        <v>80.6923164137043</v>
+      </c>
     </row>
     <row r="118" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="2" t="n">
@@ -32221,6 +33068,18 @@
       <c r="C118" s="2" t="n">
         <v>105.537390943414</v>
       </c>
+      <c r="D118" s="19" t="n">
+        <f aca="false">$D$69*(C117/AVERAGE($C$66:$C$69))</f>
+        <v>84.6847600674328</v>
+      </c>
+      <c r="E118" s="2" t="n">
+        <f aca="false">$C$98/C118</f>
+        <v>0.929367620302028</v>
+      </c>
+      <c r="F118" s="2" t="n">
+        <f aca="false">E118*D118</f>
+        <v>78.7032739397182</v>
+      </c>
     </row>
     <row r="119" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="2" t="n">
@@ -32232,6 +33091,18 @@
       <c r="C119" s="2" t="n">
         <v>105.472891746476</v>
       </c>
+      <c r="D119" s="19" t="n">
+        <f aca="false">$D$69*(C118/AVERAGE($C$66:$C$69))</f>
+        <v>84.8734402342624</v>
+      </c>
+      <c r="E119" s="2" t="n">
+        <f aca="false">$C$99/C119</f>
+        <v>0.937413310710079</v>
+      </c>
+      <c r="F119" s="2" t="n">
+        <f aca="false">E119*D119</f>
+        <v>79.5614926013539</v>
+      </c>
     </row>
     <row r="120" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="2" t="n">
@@ -32243,6 +33114,18 @@
       <c r="C120" s="2" t="n">
         <v>105.465077377946</v>
       </c>
+      <c r="D120" s="19" t="n">
+        <f aca="false">$D$69*(C119/AVERAGE($C$66:$C$69))</f>
+        <v>84.8215698148069</v>
+      </c>
+      <c r="E120" s="2" t="n">
+        <f aca="false">$C$100/C120</f>
+        <v>0.94503037417149</v>
+      </c>
+      <c r="F120" s="2" t="n">
+        <f aca="false">E120*D120</f>
+        <v>80.1589598599</v>
+      </c>
     </row>
     <row r="121" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="2" t="n">
@@ -32254,6 +33137,18 @@
       <c r="C121" s="2" t="n">
         <v>105.468976509901</v>
       </c>
+      <c r="D121" s="19" t="n">
+        <f aca="false">$D$69*(C120/AVERAGE($C$66:$C$69))</f>
+        <v>84.8152854796109</v>
+      </c>
+      <c r="E121" s="2" t="n">
+        <f aca="false">$C$101/C121</f>
+        <v>0.952947521741001</v>
+      </c>
+      <c r="F121" s="2" t="n">
+        <f aca="false">E121*D121</f>
+        <v>80.8245161035507</v>
+      </c>
     </row>
     <row r="122" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="2" t="n">
@@ -32265,6 +33160,18 @@
       <c r="C122" s="2" t="n">
         <v>105.414251920888</v>
       </c>
+      <c r="D122" s="19" t="n">
+        <f aca="false">$D$69*(C121/AVERAGE($C$66:$C$69))</f>
+        <v>84.8184211715205</v>
+      </c>
+      <c r="E122" s="2" t="n">
+        <f aca="false">$C$98/C122</f>
+        <v>0.930453255481768</v>
+      </c>
+      <c r="F122" s="2" t="n">
+        <f aca="false">E122*D122</f>
+        <v>78.919576103865</v>
+      </c>
     </row>
     <row r="123" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="2" t="n">
@@ -32276,6 +33183,18 @@
       <c r="C123" s="2" t="n">
         <v>106.152053314759</v>
       </c>
+      <c r="D123" s="19" t="n">
+        <f aca="false">$D$69*(C122/AVERAGE($C$66:$C$69))</f>
+        <v>84.7744115168055</v>
+      </c>
+      <c r="E123" s="2" t="n">
+        <f aca="false">$C$99/C123</f>
+        <v>0.931415733891254</v>
+      </c>
+      <c r="F123" s="2" t="n">
+        <f aca="false">E123*D123</f>
+        <v>78.9602207181246</v>
+      </c>
     </row>
     <row r="124" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="2" t="n">
@@ -32287,6 +33206,18 @@
       <c r="C124" s="2" t="n">
         <v>104.692229122535</v>
       </c>
+      <c r="D124" s="19" t="n">
+        <f aca="false">$D$69*(C123/AVERAGE($C$66:$C$69))</f>
+        <v>85.3677532883587</v>
+      </c>
+      <c r="E124" s="2" t="n">
+        <f aca="false">$C$100/C124</f>
+        <v>0.952006680647245</v>
+      </c>
+      <c r="F124" s="2" t="n">
+        <f aca="false">E124*D124</f>
+        <v>81.2706714423633</v>
+      </c>
     </row>
     <row r="125" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="2" t="n">
@@ -32298,6 +33229,18 @@
       <c r="C125" s="2" t="n">
         <v>104.255949350913</v>
       </c>
+      <c r="D125" s="19" t="n">
+        <f aca="false">$D$69*(C124/AVERAGE($C$66:$C$69))</f>
+        <v>84.1937589322003</v>
+      </c>
+      <c r="E125" s="2" t="n">
+        <f aca="false">$C$101/C125</f>
+        <v>0.964035150141672</v>
+      </c>
+      <c r="F125" s="2" t="n">
+        <f aca="false">E125*D125</f>
+        <v>81.1657430331955</v>
+      </c>
     </row>
     <row r="126" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="2" t="n">
@@ -32309,6 +33252,18 @@
       <c r="C126" s="2" t="n">
         <v>104.473837340587</v>
       </c>
+      <c r="D126" s="19" t="n">
+        <f aca="false">$D$69*(C125/AVERAGE($C$66:$C$69))</f>
+        <v>83.8429016219032</v>
+      </c>
+      <c r="E126" s="2" t="n">
+        <f aca="false">$C$98/C126</f>
+        <v>0.938828671088367</v>
+      </c>
+      <c r="F126" s="2" t="n">
+        <f aca="false">E126*D126</f>
+        <v>78.7141199098841</v>
+      </c>
     </row>
     <row r="127" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="2" t="n">
@@ -32320,6 +33275,18 @@
       <c r="C127" s="2" t="n">
         <v>104.987466992606</v>
       </c>
+      <c r="D127" s="19" t="n">
+        <f aca="false">$D$69*(C126/AVERAGE($C$66:$C$69))</f>
+        <v>84.0181277015329</v>
+      </c>
+      <c r="E127" s="2" t="n">
+        <f aca="false">$C$99/C127</f>
+        <v>0.941747576872134</v>
+      </c>
+      <c r="F127" s="2" t="n">
+        <f aca="false">E127*D127</f>
+        <v>79.1238681762521</v>
+      </c>
     </row>
     <row r="128" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="2" t="n">
@@ -32331,6 +33298,18 @@
       <c r="C128" s="2" t="n">
         <v>105.532277249572</v>
       </c>
+      <c r="D128" s="19" t="n">
+        <f aca="false">$D$69*(C127/AVERAGE($C$66:$C$69))</f>
+        <v>84.4311899838529</v>
+      </c>
+      <c r="E128" s="2" t="n">
+        <f aca="false">$C$100/C128</f>
+        <v>0.944428606432916</v>
+      </c>
+      <c r="F128" s="2" t="n">
+        <f aca="false">E128*D128</f>
+        <v>79.7392310959229</v>
+      </c>
     </row>
     <row r="129" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="2" t="n">
@@ -32342,6 +33321,18 @@
       <c r="C129" s="2" t="n">
         <v>106.081243504608</v>
       </c>
+      <c r="D129" s="19" t="n">
+        <f aca="false">$D$69*(C128/AVERAGE($C$66:$C$69))</f>
+        <v>84.8693277885709</v>
+      </c>
+      <c r="E129" s="2" t="n">
+        <f aca="false">$C$101/C129</f>
+        <v>0.947447413560006</v>
+      </c>
+      <c r="F129" s="2" t="n">
+        <f aca="false">E129*D129</f>
+        <v>80.4092251038578</v>
+      </c>
     </row>
     <row r="130" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="2" t="n">
@@ -32353,6 +33344,18 @@
       <c r="C130" s="2" t="n">
         <v>107.228391653468</v>
       </c>
+      <c r="D130" s="19" t="n">
+        <f aca="false">$D$69*(C129/AVERAGE($C$66:$C$69))</f>
+        <v>85.3108078575865</v>
+      </c>
+      <c r="E130" s="2" t="n">
+        <f aca="false">$C$98/C130</f>
+        <v>0.914711415153389</v>
+      </c>
+      <c r="F130" s="2" t="n">
+        <f aca="false">E130*D130</f>
+        <v>78.0347697832917</v>
+      </c>
     </row>
     <row r="131" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="2" t="n">
@@ -32364,6 +33367,18 @@
       <c r="C131" s="2" t="n">
         <v>108.665438636281</v>
       </c>
+      <c r="D131" s="19" t="n">
+        <f aca="false">$D$69*(C130/AVERAGE($C$66:$C$69))</f>
+        <v>86.2333473384451</v>
+      </c>
+      <c r="E131" s="2" t="n">
+        <f aca="false">$C$99/C131</f>
+        <v>0.90987248460081</v>
+      </c>
+      <c r="F131" s="2" t="n">
+        <f aca="false">E131*D131</f>
+        <v>78.4613499982757</v>
+      </c>
     </row>
     <row r="132" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="2" t="n">
@@ -32375,6 +33390,18 @@
       <c r="C132" s="2" t="n">
         <v>109.662008713931</v>
       </c>
+      <c r="D132" s="19" t="n">
+        <f aca="false">$D$69*(C131/AVERAGE($C$66:$C$69))</f>
+        <v>87.3890242044291</v>
+      </c>
+      <c r="E132" s="2" t="n">
+        <f aca="false">$C$100/C132</f>
+        <v>0.908862628957517</v>
+      </c>
+      <c r="F132" s="2" t="n">
+        <f aca="false">E132*D132</f>
+        <v>79.4246182804694</v>
+      </c>
     </row>
     <row r="133" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="2" t="n">
@@ -32386,6 +33413,18 @@
       <c r="C133" s="2" t="n">
         <v>110.114154178387</v>
       </c>
+      <c r="D133" s="19" t="n">
+        <f aca="false">$D$69*(C132/AVERAGE($C$66:$C$69))</f>
+        <v>88.1904684145672</v>
+      </c>
+      <c r="E133" s="2" t="n">
+        <f aca="false">$C$101/C133</f>
+        <v>0.912747326041734</v>
+      </c>
+      <c r="F133" s="2" t="n">
+        <f aca="false">E133*D133</f>
+        <v>80.4956142277642</v>
+      </c>
     </row>
     <row r="134" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="2" t="n">
@@ -32397,6 +33436,18 @@
       <c r="C134" s="2" t="n">
         <v>110.397594317166</v>
       </c>
+      <c r="D134" s="19" t="n">
+        <f aca="false">$D$69*(C133/AVERAGE($C$66:$C$69))</f>
+        <v>88.5540849556969</v>
+      </c>
+      <c r="E134" s="2" t="n">
+        <f aca="false">$C$98/C134</f>
+        <v>0.888452637764719</v>
+      </c>
+      <c r="F134" s="2" t="n">
+        <f aca="false">E134*D134</f>
+        <v>78.6761103637299</v>
+      </c>
     </row>
     <row r="135" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="2" t="n">
@@ -32408,6 +33459,18 @@
       <c r="C135" s="2" t="n">
         <v>110.872665883349</v>
       </c>
+      <c r="D135" s="19" t="n">
+        <f aca="false">$D$69*(C134/AVERAGE($C$66:$C$69))</f>
+        <v>88.782028241613</v>
+      </c>
+      <c r="E135" s="2" t="n">
+        <f aca="false">$C$99/C135</f>
+        <v>0.891758954783809</v>
+      </c>
+      <c r="F135" s="2" t="n">
+        <f aca="false">E135*D135</f>
+        <v>79.1721687083274</v>
+      </c>
     </row>
     <row r="136" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="2" t="n">
@@ -32419,6 +33482,18 @@
       <c r="C136" s="2" t="n">
         <v>112.169848642022</v>
       </c>
+      <c r="D136" s="19" t="n">
+        <f aca="false">$D$69*(C135/AVERAGE($C$66:$C$69))</f>
+        <v>89.1640820124992</v>
+      </c>
+      <c r="E136" s="2" t="n">
+        <f aca="false">$C$100/C136</f>
+        <v>0.888542712173787</v>
+      </c>
+      <c r="F136" s="2" t="n">
+        <f aca="false">E136*D136</f>
+        <v>79.2260952598721</v>
+      </c>
     </row>
     <row r="137" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="2" t="n">
@@ -32430,6 +33505,18 @@
       <c r="C137" s="2" t="n">
         <v>111.881688987881</v>
       </c>
+      <c r="D137" s="19" t="n">
+        <f aca="false">$D$69*(C136/AVERAGE($C$66:$C$69))</f>
+        <v>90.2072797110304</v>
+      </c>
+      <c r="E137" s="2" t="n">
+        <f aca="false">$C$101/C137</f>
+        <v>0.89832751627978</v>
+      </c>
+      <c r="F137" s="2" t="n">
+        <f aca="false">E137*D137</f>
+        <v>81.0356815331653</v>
+      </c>
     </row>
     <row r="138" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="2" t="n">
@@ -32441,6 +33528,18 @@
       <c r="C138" s="2" t="n">
         <v>112.031841115164</v>
       </c>
+      <c r="D138" s="19" t="n">
+        <f aca="false">$D$69*(C137/AVERAGE($C$66:$C$69))</f>
+        <v>89.9755409787665</v>
+      </c>
+      <c r="E138" s="2" t="n">
+        <f aca="false">$C$98/C138</f>
+        <v>0.875492475153919</v>
+      </c>
+      <c r="F138" s="2" t="n">
+        <f aca="false">E138*D138</f>
+        <v>78.7729090748131</v>
+      </c>
     </row>
     <row r="139" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="2" t="n">
@@ -32452,6 +33551,18 @@
       <c r="C139" s="2" t="n">
         <v>113.260097496806</v>
       </c>
+      <c r="D139" s="19" t="n">
+        <f aca="false">$D$69*(C138/AVERAGE($C$66:$C$69))</f>
+        <v>90.0962937042895</v>
+      </c>
+      <c r="E139" s="2" t="n">
+        <f aca="false">$C$99/C139</f>
+        <v>0.87296139441358</v>
+      </c>
+      <c r="F139" s="2" t="n">
+        <f aca="false">E139*D139</f>
+        <v>78.650586183592</v>
+      </c>
     </row>
     <row r="140" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="2" t="n">
@@ -32463,6 +33574,18 @@
       <c r="C140" s="2" t="n">
         <v>113.771246610086</v>
       </c>
+      <c r="D140" s="19" t="n">
+        <f aca="false">$D$69*(C139/AVERAGE($C$66:$C$69))</f>
+        <v>91.0840606337897</v>
+      </c>
+      <c r="E140" s="2" t="n">
+        <f aca="false">$C$100/C140</f>
+        <v>0.876035944987788</v>
+      </c>
+      <c r="F140" s="2" t="n">
+        <f aca="false">E140*D140</f>
+        <v>79.792911130647</v>
+      </c>
     </row>
     <row r="141" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="2" t="n">
@@ -32473,6 +33596,18 @@
       </c>
       <c r="C141" s="2" t="n">
         <v>113.148518059142</v>
+      </c>
+      <c r="D141" s="19" t="n">
+        <f aca="false">$D$69*(C140/AVERAGE($C$66:$C$69))</f>
+        <v>91.4951280604994</v>
+      </c>
+      <c r="E141" s="2" t="n">
+        <f aca="false">$C$101/C141</f>
+        <v>0.888269696410305</v>
+      </c>
+      <c r="F141" s="2" t="n">
+        <f aca="false">E141*D141</f>
+        <v>81.2723496253218</v>
       </c>
     </row>
   </sheetData>
@@ -32483,6 +33618,7 @@
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
-  <legacyDrawing r:id="rId2"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>